<commit_message>
Final commit of master thesis
</commit_message>
<xml_diff>
--- a/project/Train data/TRAXX_AC3_Training_allCabs_8class_cnt250.xlsx
+++ b/project/Train data/TRAXX_AC3_Training_allCabs_8class_cnt250.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\OneDrive\Masterarbeit\FTS Daten\Training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Masterarbeit Code\control_element_classification\project\Train data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B8825D-5EE1-498A-BA58-07EC0988387C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9623B4DE-2884-4434-B86B-450A3FDEED96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B4F8F2C-B747-4AAD-A2F5-B6A6451F8155}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="14370" windowHeight="14745" xr2:uid="{9B4F8F2C-B747-4AAD-A2F5-B6A6451F8155}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4584,87 +4584,7 @@
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -27020,6 +26940,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdSecurityGroups xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
+    <MigrationWizIdPermissions xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
+    <_activity xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
+    <MigrationWizIdPermissionLevels xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
+    <MigrationWizId xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
+    <MigrationWizIdDocumentLibraryPermissions xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007051E9AA93382B418BEC4198347C7550" ma:contentTypeVersion="23" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae4185827d492789805aecd68fb30589">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0935a800-1f2a-43fd-bd04-bde7fe816747" xmlns:ns4="b36ee72d-ae3f-4bd9-b38d-8bf34fa6f818" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0a45c92692b36d6ecab2a69ce0446f07" ns3:_="" ns4:_="">
     <xsd:import namespace="0935a800-1f2a-43fd-bd04-bde7fe816747"/>
@@ -27302,19 +27235,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdSecurityGroups xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
-    <MigrationWizIdPermissions xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
-    <_activity xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
-    <MigrationWizIdPermissionLevels xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
-    <MigrationWizId xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
-    <MigrationWizIdDocumentLibraryPermissions xmlns="0935a800-1f2a-43fd-bd04-bde7fe816747" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -27325,6 +27245,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2006733-797B-4E3E-96E0-B838FEF166B9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="0935a800-1f2a-43fd-bd04-bde7fe816747"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="b36ee72d-ae3f-4bd9-b38d-8bf34fa6f818"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9272C589-7E9A-4F1B-BC40-98C0C4C9F842}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27343,23 +27280,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2006733-797B-4E3E-96E0-B838FEF166B9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="0935a800-1f2a-43fd-bd04-bde7fe816747"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="b36ee72d-ae3f-4bd9-b38d-8bf34fa6f818"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5403A3E9-C18A-42EA-B3DC-A53EC52DE43D}">
   <ds:schemaRefs>

</xml_diff>